<commit_message>
Generate BST packages from app/data and app/templates
Triggered by: 70c9096afc420eee3cf5f3bd245ab710632c6bf9
</commit_message>
<xml_diff>
--- a/examples/se-latest/Fixedassets.xlsx
+++ b/examples/se-latest/Fixedassets.xlsx
@@ -1410,6 +1410,16 @@
             <v>0.14</v>
           </cell>
         </row>
+        <row r="8">
+          <cell r="E8">
+            <v>12000</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="G8">
+            <v>3000</v>
+          </cell>
+        </row>
         <row r="13">
           <cell r="G13">
             <v>0</v>
@@ -1732,11 +1742,11 @@
       </c>
       <c r="R1" s="13" t="n">
         <f aca="false">R57+R110</f>
-        <v>3360</v>
+        <v>3000</v>
       </c>
       <c r="S1" s="13" t="n">
         <f aca="false">S57+S110</f>
-        <v>20640</v>
+        <v>21000</v>
       </c>
       <c r="T1" s="16"/>
       <c r="U1" s="17" t="s">
@@ -1756,7 +1766,7 @@
       </c>
       <c r="Y1" s="13" t="n">
         <f aca="false">Y57+Y110</f>
-        <v>8140</v>
+        <v>8500</v>
       </c>
       <c r="Z1" s="13" t="n">
         <f aca="false">Z57+Z110</f>
@@ -3622,7 +3632,7 @@
       <c r="C37" s="69"/>
       <c r="D37" s="70" t="n">
         <f aca="false">[1]Admin!$E$8</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="E37" s="50"/>
       <c r="F37" s="50"/>
@@ -3695,12 +3705,12 @@
       <c r="P38" s="48"/>
       <c r="Q38" s="47"/>
       <c r="R38" s="47" t="n">
-        <f aca="false">IF(O38&gt;0,O38*R$4*(1-M38)," ")</f>
-        <v>3360</v>
+        <f aca="false">IF(O38&gt;0,MIN(O38*R$4*(1-M38),[1]Admin!$G$8*(1-M38))," ")</f>
+        <v>3000</v>
       </c>
       <c r="S38" s="47" t="n">
         <f aca="false">IF(O38&gt;0,O38-R38," ")</f>
-        <v>20640</v>
+        <v>21000</v>
       </c>
       <c r="T38" s="47"/>
       <c r="U38" s="54" t="n">
@@ -3719,7 +3729,7 @@
       </c>
       <c r="Y38" s="47" t="n">
         <f aca="false">IF((U38+V38)&gt;0,IF(V38&lt;S38,(S38-V38)*(1-M38)," ")," ")</f>
-        <v>8140</v>
+        <v>8500</v>
       </c>
       <c r="Z38" s="47" t="str">
         <f aca="false">IF((U38+V38)&gt;0,IF(V38&gt;S38,(V38-S38)*(1-M38)," ")," ")</f>
@@ -3763,7 +3773,7 @@
       <c r="P39" s="48"/>
       <c r="Q39" s="47"/>
       <c r="R39" s="47" t="str">
-        <f aca="false">IF(O39&gt;0,O39*R$4*(1-M39)," ")</f>
+        <f aca="false">IF(O39&gt;0,MIN(O39*R$4*(1-M39),[1]Admin!$G$8*(1-M39))," ")</f>
         <v> </v>
       </c>
       <c r="S39" s="47" t="str">
@@ -3827,7 +3837,7 @@
       <c r="P40" s="48"/>
       <c r="Q40" s="47"/>
       <c r="R40" s="47" t="str">
-        <f aca="false">IF(O40&gt;0,O40*R$4*(1-M40)," ")</f>
+        <f aca="false">IF(O40&gt;0,MIN(O40*R$4*(1-M40),[1]Admin!$G$8*(1-M40))," ")</f>
         <v> </v>
       </c>
       <c r="S40" s="47" t="str">
@@ -3891,7 +3901,7 @@
       <c r="P41" s="48"/>
       <c r="Q41" s="47"/>
       <c r="R41" s="47" t="str">
-        <f aca="false">IF(O41&gt;0,O41*R$4*(1-M41)," ")</f>
+        <f aca="false">IF(O41&gt;0,MIN(O41*R$4*(1-M41),[1]Admin!$G$8*(1-M41))," ")</f>
         <v> </v>
       </c>
       <c r="S41" s="47" t="str">
@@ -3955,7 +3965,7 @@
       <c r="P42" s="48"/>
       <c r="Q42" s="47"/>
       <c r="R42" s="47" t="str">
-        <f aca="false">IF(O42&gt;0,O42*R$4*(1-M42)," ")</f>
+        <f aca="false">IF(O42&gt;0,MIN(O42*R$4*(1-M42),[1]Admin!$G$8*(1-M42))," ")</f>
         <v> </v>
       </c>
       <c r="S42" s="47" t="str">
@@ -3991,7 +4001,7 @@
       <c r="C43" s="69"/>
       <c r="D43" s="70" t="n">
         <f aca="false">[1]Admin!$E$8</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="E43" s="50"/>
       <c r="F43" s="50"/>
@@ -4053,7 +4063,7 @@
       <c r="P44" s="48"/>
       <c r="Q44" s="47"/>
       <c r="R44" s="47" t="str">
-        <f aca="false">IF(O44&gt;0,O44*R$4*(1-M44)," ")</f>
+        <f aca="false">IF(O44&gt;0,MIN(O44*R$4*(1-M44),[1]Admin!$G$8*(1-M44))," ")</f>
         <v> </v>
       </c>
       <c r="S44" s="47" t="str">
@@ -4117,7 +4127,7 @@
       <c r="P45" s="48"/>
       <c r="Q45" s="47"/>
       <c r="R45" s="47" t="str">
-        <f aca="false">IF(O45&gt;0,O45*R$4*(1-M45)," ")</f>
+        <f aca="false">IF(O45&gt;0,MIN(O45*R$4*(1-M45),[1]Admin!$G$8*(1-M45))," ")</f>
         <v> </v>
       </c>
       <c r="S45" s="47" t="str">
@@ -4181,7 +4191,7 @@
       <c r="P46" s="48"/>
       <c r="Q46" s="47"/>
       <c r="R46" s="47" t="str">
-        <f aca="false">IF(O46&gt;0,O46*R$4*(1-M46)," ")</f>
+        <f aca="false">IF(O46&gt;0,MIN(O46*R$4*(1-M46),[1]Admin!$G$8*(1-M46))," ")</f>
         <v> </v>
       </c>
       <c r="S46" s="47" t="str">
@@ -4245,7 +4255,7 @@
       <c r="P47" s="48"/>
       <c r="Q47" s="47"/>
       <c r="R47" s="47" t="str">
-        <f aca="false">IF(O47&gt;0,O47*R$4*(1-M47)," ")</f>
+        <f aca="false">IF(O47&gt;0,MIN(O47*R$4*(1-M47),[1]Admin!$G$8*(1-M47))," ")</f>
         <v> </v>
       </c>
       <c r="S47" s="47" t="str">
@@ -4309,7 +4319,7 @@
       <c r="P48" s="48"/>
       <c r="Q48" s="47"/>
       <c r="R48" s="47" t="str">
-        <f aca="false">IF(O48&gt;0,O48*R$4*(1-M48)," ")</f>
+        <f aca="false">IF(O48&gt;0,MIN(O48*R$4*(1-M48),[1]Admin!$G$8*(1-M48))," ")</f>
         <v> </v>
       </c>
       <c r="S48" s="47" t="str">
@@ -4734,11 +4744,11 @@
       </c>
       <c r="R55" s="61" t="n">
         <f aca="false">SUM(R38:R54)</f>
-        <v>3360</v>
+        <v>3000</v>
       </c>
       <c r="S55" s="61" t="n">
         <f aca="false">SUM(S38:S54)</f>
-        <v>20640</v>
+        <v>21000</v>
       </c>
       <c r="T55" s="50"/>
       <c r="U55" s="49"/>
@@ -4756,7 +4766,7 @@
       </c>
       <c r="Y55" s="61" t="n">
         <f aca="false">SUM(Y38:Y54)</f>
-        <v>8140</v>
+        <v>8500</v>
       </c>
       <c r="Z55" s="61" t="n">
         <f aca="false">SUM(Z38:Z54)</f>
@@ -4843,11 +4853,11 @@
       </c>
       <c r="R57" s="74" t="n">
         <f aca="false">R11+R19+R27+R35+R55</f>
-        <v>3360</v>
+        <v>3000</v>
       </c>
       <c r="S57" s="74" t="n">
         <f aca="false">S11+S19+S27+S35+S55</f>
-        <v>20640</v>
+        <v>21000</v>
       </c>
       <c r="T57" s="47"/>
       <c r="U57" s="49"/>
@@ -4865,7 +4875,7 @@
       </c>
       <c r="Y57" s="74" t="n">
         <f aca="false">Y11+Y19+Y27+Y35+Y55</f>
-        <v>8140</v>
+        <v>8500</v>
       </c>
       <c r="Z57" s="74" t="n">
         <f aca="false">Z11+Z19+Z27+Z35+Z55</f>
@@ -6602,7 +6612,7 @@
       <c r="C90" s="69"/>
       <c r="D90" s="70" t="n">
         <f aca="false">D37</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="E90" s="50"/>
       <c r="F90" s="50"/>
@@ -6664,7 +6674,7 @@
       <c r="P91" s="48"/>
       <c r="Q91" s="47"/>
       <c r="R91" s="47" t="str">
-        <f aca="false">IF(E91&gt;0,E91*R$4*(1-M91)," ")</f>
+        <f aca="false">IF(E91&gt;0,MIN(E91*R$4*(1-M91),[1]Admin!$G$8*(1-M91))," ")</f>
         <v> </v>
       </c>
       <c r="S91" s="47" t="str">
@@ -6725,7 +6735,7 @@
       <c r="P92" s="48"/>
       <c r="Q92" s="47"/>
       <c r="R92" s="47" t="str">
-        <f aca="false">IF(E92&gt;0,E92*R$4*(1-M92)," ")</f>
+        <f aca="false">IF(E92&gt;0,MIN(E92*R$4*(1-M92),[1]Admin!$G$8*(1-M92))," ")</f>
         <v> </v>
       </c>
       <c r="S92" s="47" t="str">
@@ -6786,7 +6796,7 @@
       <c r="P93" s="48"/>
       <c r="Q93" s="47"/>
       <c r="R93" s="47" t="str">
-        <f aca="false">IF(E93&gt;0,E93*R$4*(1-M93)," ")</f>
+        <f aca="false">IF(E93&gt;0,MIN(E93*R$4*(1-M93),[1]Admin!$G$8*(1-M93))," ")</f>
         <v> </v>
       </c>
       <c r="S93" s="47" t="str">
@@ -6847,7 +6857,7 @@
       <c r="P94" s="48"/>
       <c r="Q94" s="47"/>
       <c r="R94" s="47" t="str">
-        <f aca="false">IF(E94&gt;0,E94*R$4*(1-M94)," ")</f>
+        <f aca="false">IF(E94&gt;0,MIN(E94*R$4*(1-M94),[1]Admin!$G$8*(1-M94))," ")</f>
         <v> </v>
       </c>
       <c r="S94" s="47" t="str">
@@ -6908,7 +6918,7 @@
       <c r="P95" s="48"/>
       <c r="Q95" s="47"/>
       <c r="R95" s="47" t="str">
-        <f aca="false">IF(E95&gt;0,E95*R$4*(1-M95)," ")</f>
+        <f aca="false">IF(E95&gt;0,MIN(E95*R$4*(1-M95),[1]Admin!$G$8*(1-M95))," ")</f>
         <v> </v>
       </c>
       <c r="S95" s="47" t="str">
@@ -6945,7 +6955,7 @@
       <c r="C96" s="83"/>
       <c r="D96" s="70" t="n">
         <f aca="false">D43</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="E96" s="50"/>
       <c r="F96" s="50"/>
@@ -7004,7 +7014,7 @@
       <c r="P97" s="48"/>
       <c r="Q97" s="47"/>
       <c r="R97" s="47" t="str">
-        <f aca="false">IF(E97&gt;0,E97*R$4*(1-M97)," ")</f>
+        <f aca="false">IF(E97&gt;0,MIN(E97*R$4*(1-M97),[1]Admin!$G$8*(1-M97))," ")</f>
         <v> </v>
       </c>
       <c r="S97" s="47" t="str">
@@ -7065,7 +7075,7 @@
       <c r="P98" s="48"/>
       <c r="Q98" s="47"/>
       <c r="R98" s="47" t="str">
-        <f aca="false">IF(E98&gt;0,E98*R$4*(1-M98)," ")</f>
+        <f aca="false">IF(E98&gt;0,MIN(E98*R$4*(1-M98),[1]Admin!$G$8*(1-M98))," ")</f>
         <v> </v>
       </c>
       <c r="S98" s="47" t="str">
@@ -7126,7 +7136,7 @@
       <c r="P99" s="48"/>
       <c r="Q99" s="47"/>
       <c r="R99" s="47" t="str">
-        <f aca="false">IF(E99&gt;0,E99*R$4*(1-M99)," ")</f>
+        <f aca="false">IF(E99&gt;0,MIN(E99*R$4*(1-M99),[1]Admin!$G$8*(1-M99))," ")</f>
         <v> </v>
       </c>
       <c r="S99" s="47" t="str">
@@ -7187,7 +7197,7 @@
       <c r="P100" s="48"/>
       <c r="Q100" s="47"/>
       <c r="R100" s="47" t="str">
-        <f aca="false">IF(E100&gt;0,E100*R$4*(1-M100)," ")</f>
+        <f aca="false">IF(E100&gt;0,MIN(E100*R$4*(1-M100),[1]Admin!$G$8*(1-M100))," ")</f>
         <v> </v>
       </c>
       <c r="S100" s="47" t="str">
@@ -7248,7 +7258,7 @@
       <c r="P101" s="48"/>
       <c r="Q101" s="47"/>
       <c r="R101" s="47" t="str">
-        <f aca="false">IF(E101&gt;0,E101*R$4*(1-M101)," ")</f>
+        <f aca="false">IF(E101&gt;0,MIN(E101*R$4*(1-M101),[1]Admin!$G$8*(1-M101))," ")</f>
         <v> </v>
       </c>
       <c r="S101" s="47" t="str">

</xml_diff>